<commit_message>
KAVIX: gerador da campanha 3 (300 reels, 10 formatos) e hashtags novas nas legendas
- campanha3.py: jogos (ficha, escada, escolha, cronômetro), skins (abrindo,
  kit, top3) e ranked (patentes, vaga no top, duelo online)
- gerar_videos.py: opção para esconder o @perfil e a barra de progresso
- legendas das campanhas 1 e 2: #roblox #jogosonline #jogos #mobile + virais

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UYA8DmSnk7TrkabtFVHiQr
</commit_message>
<xml_diff>
--- a/promo/kavix/campanha2/youtube_reverso/calendario_youtube_reverso.xlsx
+++ b/promo/kavix/campanha2/youtube_reverso/calendario_youtube_reverso.xlsx
@@ -68,12 +68,8 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -442,17 +438,17 @@
   <dimension ref="A1:K101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="27" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="50" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" style="4" min="1" max="1"/>
+    <col width="9" customWidth="1" style="4" min="2" max="2"/>
+    <col width="6" customWidth="1" style="4" min="3" max="3"/>
+    <col width="12" customWidth="1" style="4" min="4" max="4"/>
+    <col width="7" customWidth="1" style="4" min="5" max="5"/>
+    <col width="27" customWidth="1" style="4" min="6" max="6"/>
+    <col width="34" customWidth="1" style="4" min="7" max="7"/>
+    <col width="40" customWidth="1" style="4" min="8" max="8"/>
+    <col width="50" customWidth="1" style="4" min="9" max="9"/>
+    <col width="60" customWidth="1" style="4" min="10" max="10"/>
+    <col width="12" customWidth="1" style="4" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -513,41 +509,41 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>2026-10-14T09:00:00-03:00</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>videos/100_desafio_equilibrio.mp4</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/100_desafio_equilibrio.mp4</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>DESAFIO: faz 10 pontos no Equilíbrio 😤 manda print nos comentários 📸 #shorts</t>
         </is>
@@ -556,51 +552,51 @@
         <is>
           <t>DESAFIO: faz 10 pontos no Equilíbrio 😤 manda print nos comentários 📸
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #fyp #trend #foryou #robloxbrasil #robloxedit #jogosgratis #jogosonline #shorts</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #trend #foryou #robloxbrasil #robloxedit #jogosgratis #shorts</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="3" t="n">
         <v>99</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>2026-10-14T12:30:00-03:00</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>videos/099_meme_testar.mp4</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/099_meme_testar.mp4</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>eu: vou só testar / eu 2 horas depois: 😭 #shorts</t>
         </is>
@@ -609,51 +605,51 @@
         <is>
           <t>eu: vou só testar / eu 2 horas depois: 😭
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #fyp #paravoce #explore #robloxgames #roblox #robloxfyp #minigames #jogosonline #shorts</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #paravoce #explore #robloxgames #robloxfyp #minigames #shorts</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="3" t="n">
         <v>98</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>2026-10-14T17:00:00-03:00</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>videos/098_tutorial_passos_8.mp4</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/098_tutorial_passos_8.mp4</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>como jogar em 3 passos 👇 tá entediado? 😴 → kavixbrasil.com.br 🔗 → problema resol #shorts</t>
         </is>
@@ -662,51 +658,51 @@
         <is>
           <t>como jogar em 3 passos 👇 tá entediado? 😴 → kavixbrasil.com.br 🔗 → problema resolvido 😎
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #viral #foryou #fyp #robloxbrasil #robloxgames #jogosgratis #minigames #shorts</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #foryou #fyp #robloxbrasil #robloxgames #jogosgratis #minigames #shorts</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>97</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>2026-10-14T20:30:00-03:00</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>videos/097_pergunta_precisa_de_cadastro_pra_jogar.mp4</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/097_pergunta_precisa_de_cadastro_pra_jogar.mp4</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>precisa de cadastro pra jogar? cadastro rápido e ainda ganha itens 🎁 #shorts</t>
         </is>
@@ -715,10 +711,10 @@
         <is>
           <t>precisa de cadastro pra jogar? cadastro rápido e ainda ganha itens 🎁
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #foryou #trend #explore #robloxgames #robloxbrasil #robloxfyp #jogosgratis #minigames #shorts</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #foryou #trend #explore #robloxgames #robloxbrasil #robloxfyp #shorts</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -764,11 +760,11 @@
           <t>DESAFIO: faz 25 pontos no Troca Cor 😤 comenta teu recorde 👇 #shorts</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>DESAFIO: faz 25 pontos no Troca Cor 😤 comenta teu recorde 👇
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #fyp #foryou #trend #roblox #robloxgames #mobilegames #jogosgratis #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #foryou #trend #robloxgames #mobilegames #jogosgratis #shorts</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -817,11 +813,11 @@
           <t>skin do dia: Visor Cyber (Épico) ✨ #shorts</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>skin do dia: Visor Cyber (Épico) ✨
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #paravoce #viralvideo #fyp #robloxgames #robloxbrasil #robloxfyp #jogosgratis #minigames #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #paravoce #viralvideo #fyp #robloxgames #robloxbrasil #robloxfyp #shorts</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -870,11 +866,11 @@
           <t>DESAFIO: faz 10 pontos no Cobrinha 😤 manda print nos comentários 📸 #shorts</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>DESAFIO: faz 10 pontos no Cobrinha 😤 manda print nos comentários 📸
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #explore #paravoce #viralvideo #robloxbrasil #robloxgames #mobilegames #jogosonline #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #explore #paravoce #viralvideo #robloxbrasil #robloxgames #shorts</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -923,11 +919,11 @@
           <t>Ninja ou Óculos Dourados? qual é mais bonita? 👇 #shorts</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Ninja ou Óculos Dourados? qual é mais bonita? 👇
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #explore #trend #fyp #robloxgames #robloxedit #robloxfyp #gamerbrasil #jogosgratis #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #explore #trend #fyp #robloxgames #robloxedit #robloxfyp #shorts</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -937,41 +933,41 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="3" t="n">
         <v>92</v>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>2026-10-16T09:00:00-03:00</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>videos/092_skin_do_dia_aura_de_fogo.mp4</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/092_skin_do_dia_aura_de_fogo.mp4</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>skin do dia: Aura de Fogo (Épico) ✨ #shorts</t>
         </is>
@@ -980,51 +976,51 @@
         <is>
           <t>skin do dia: Aura de Fogo (Épico) ✨
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #fyp #explore #paravoce #robloxbrasil #robloxgames #jogosgratis #jogosonline #shorts</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #explore #paravoce #robloxbrasil #robloxgames #jogosgratis #shorts</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="3" t="n">
         <v>91</v>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C11" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>2026-10-16T12:30:00-03:00</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>videos/091_tier_list_tier_list_dos_jogos_mais_dificeis.mp4</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/091_tier_list_tier_list_dos_jogos_mais_dificeis.mp4</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>tier list dos jogos mais difíceis 🔥 concorda? #shorts</t>
         </is>
@@ -1033,51 +1029,51 @@
         <is>
           <t>tier list dos jogos mais difíceis 🔥 concorda?
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #trend #foryou #explore #robloxedit #robloxfyp #roblox #jogosgratis #mobilegames #shorts</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #trend #foryou #explore #robloxedit #robloxfyp #jogosgratis #shorts</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="3" t="n">
         <v>90</v>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C12" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>2026-10-16T17:00:00-03:00</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>videos/090_pergunta_e_de_graca.mp4</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/090_pergunta_e_de_graca.mp4</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>é de graça? é! joga de graça 🎮 #shorts</t>
         </is>
@@ -1086,51 +1082,51 @@
         <is>
           <t>é de graça? é! joga de graça 🎮
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #foryou #fyp #viralvideo #robloxbrasil #robloxgames #minigames #mobilegames #shorts</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #foryou #fyp #viralvideo #robloxbrasil #robloxgames #minigames #mobilegames #shorts</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" s="3" t="n">
         <v>89</v>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="C13" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>2026-10-16T20:30:00-03:00</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>videos/089_meme_empilha.mp4</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/089_meme_empilha.mp4</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>ninguém: / eu no Empilha: 😭 #shorts</t>
         </is>
@@ -1139,10 +1135,10 @@
         <is>
           <t>ninguém: / eu no Empilha: 😭
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #viralvideo #paravoce #fyp #roblox #robloxgames #robloxbrasil #jogosgratis #gamerbrasil #shorts</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #viralvideo #paravoce #fyp #robloxgames #robloxbrasil #jogosgratis #shorts</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -1188,11 +1184,11 @@
           <t>DESAFIO: faz 15 pontos no Reflexo 😤 marca quem consegue 👇 #shorts</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>DESAFIO: faz 15 pontos no Reflexo 😤 marca quem consegue 👇
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #explore #fyp #viralvideo #robloxgames #robloxbrasil #gamerbrasil #jogosgratis #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #explore #fyp #viralvideo #robloxgames #robloxbrasil #gamerbrasil #shorts</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1241,11 +1237,11 @@
           <t>como jogar em 3 passos 👇 salva esse vídeo 📌 → entra no site depois 🔗 → me agrade #shorts</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>como jogar em 3 passos 👇 salva esse vídeo 📌 → entra no site depois 🔗 → me agradece 😎
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #explore #foryou #viral #robloxedit #roblox #robloxgames #jogosdecelular #minigames #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #fyp #explore #foryou #viral #robloxedit #robloxgames #jogosdecelular #minigames #shorts</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1294,11 +1290,11 @@
           <t>Auréola ou Cor Ouro? qual é mais bonita? 👇 #shorts</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>Auréola ou Cor Ouro? qual é mais bonita? 👇
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #viral #trend #fyp #robloxgames #robloxfyp #minigames #jogosdecelular #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #trend #fyp #robloxgames #robloxfyp #minigames #jogosdecelular #shorts</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1347,11 +1343,11 @@
           <t>DESAFIO: faz 20 pontos no Gravidade 😤 duvido tu bater 😤 #shorts</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>DESAFIO: faz 20 pontos no Gravidade 😤 duvido tu bater 😤
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #paravoce #explore #viralvideo #robloxfyp #robloxedit #roblox #jogosgratis #minigames #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #paravoce #explore #viralvideo #robloxfyp #robloxedit #shorts</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1361,41 +1357,41 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B18" s="3" t="n">
         <v>84</v>
       </c>
-      <c r="C18" s="2" t="n">
+      <c r="C18" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>18/10/2026</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>2026-10-18T09:00:00-03:00</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>videos/084_meme_fila.mp4</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/084_meme_fila.mp4</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>quando a fila não anda / eu tranquilão: 😭 #shorts</t>
         </is>
@@ -1404,51 +1400,51 @@
         <is>
           <t>quando a fila não anda / eu tranquilão: 😭
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #viral #fyp #viralvideo #robloxfyp #robloxgames #jogosdecelular #mobilegames #shorts</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #viralvideo #robloxfyp #robloxgames #jogosdecelular #mobilegames #shorts</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B19" s="3" t="n">
         <v>83</v>
       </c>
-      <c r="C19" s="2" t="n">
+      <c r="C19" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>18/10/2026</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>2026-10-18T12:30:00-03:00</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>videos/083_desafio_espelho.mp4</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/083_desafio_espelho.mp4</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>DESAFIO: faz 15 pontos no Espelho 😤 marca quem consegue 👇 #shorts</t>
         </is>
@@ -1457,51 +1453,51 @@
         <is>
           <t>DESAFIO: faz 15 pontos no Espelho 😤 marca quem consegue 👇
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #foryou #paravoce #viralvideo #roblox #robloxfyp #robloxedit #minigames #mobilegames #shorts</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #foryou #paravoce #viralvideo #robloxfyp #robloxedit #minigames #shorts</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B20" s="3" t="n">
         <v>82</v>
       </c>
-      <c r="C20" s="2" t="n">
+      <c r="C20" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>18/10/2026</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>2026-10-18T17:00:00-03:00</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>videos/082_skin_do_dia_aura_dourada.mp4</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/082_skin_do_dia_aura_dourada.mp4</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>skin do dia: Aura Dourada (Épico) ✨ #shorts</t>
         </is>
@@ -1510,51 +1506,51 @@
         <is>
           <t>skin do dia: Aura Dourada (Épico) ✨
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #explore #viral #fyp #robloxbrasil #robloxedit #gamerbrasil #mobilegames #shorts</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #explore #viral #fyp #robloxbrasil #robloxedit #gamerbrasil #mobilegames #shorts</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B21" s="3" t="n">
         <v>81</v>
       </c>
-      <c r="C21" s="2" t="n">
+      <c r="C21" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>18/10/2026</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>2026-10-18T20:30:00-03:00</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>videos/081_pergunta_tem_jogo_tipo_cobrinha.mp4</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/081_pergunta_tem_jogo_tipo_cobrinha.mp4</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>tem jogo tipo cobrinha? tem a própria Cobrinha 🐍 #shorts</t>
         </is>
@@ -1563,10 +1559,10 @@
         <is>
           <t>tem jogo tipo cobrinha? tem a própria Cobrinha 🐍
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #paravoce #explore #foryou #roblox #robloxgames #robloxfyp #minigames #mobilegames #shorts</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #paravoce #explore #foryou #robloxgames #robloxfyp #minigames #shorts</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -1612,11 +1608,11 @@
           <t>DESAFIO: faz 25 pontos no Três Pistas 😤 comenta teu recorde 👇 #shorts</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>DESAFIO: faz 25 pontos no Três Pistas 😤 comenta teu recorde 👇
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #paravoce #trend #foryou #robloxbrasil #roblox #gamerbrasil #jogosgratis #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #paravoce #trend #foryou #robloxbrasil #gamerbrasil #jogosgratis #shorts</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1665,11 +1661,11 @@
           <t>qual o jogo mais difícil? Fio... boa sorte 💀 #shorts</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>qual o jogo mais difícil? Fio... boa sorte 💀
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #viral #foryou #paravoce #robloxfyp #robloxedit #robloxbrasil #jogosgratis #mobilegames #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #fyp #viral #foryou #paravoce #robloxfyp #robloxedit #robloxbrasil #jogosgratis #shorts</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1718,11 +1714,11 @@
           <t>skin do dia: Chifres de Fogo (Épico) ✨ #shorts</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>skin do dia: Chifres de Fogo (Épico) ✨
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #foryou #viral #viralvideo #robloxbrasil #robloxgames #mobilegames #jogosonline #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #fyp #foryou #viral #viralvideo #robloxbrasil #robloxgames #mobilegames #shorts</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1771,11 +1767,11 @@
           <t>domingo à noite / eu descobrindo 30 jogos: 😭 #shorts</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>domingo à noite / eu descobrindo 30 jogos: 😭
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #fyp #viral #trend #roblox #robloxgames #robloxedit #minigames #jogosdecelular #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #fyp #viral #trend #robloxgames #robloxedit #minigames #jogosdecelular #shorts</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -1785,41 +1781,41 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="2" t="n">
+      <c r="B26" s="3" t="n">
         <v>76</v>
       </c>
-      <c r="C26" s="2" t="n">
+      <c r="C26" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>2026-10-20T09:00:00-03:00</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>videos/076_duelo_skins_mascarado_vs_magma.mp4</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/076_duelo_skins_mascarado_vs_magma.mp4</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>Mascarado ou Magma? qual é mais bonita? 👇 #shorts</t>
         </is>
@@ -1828,51 +1824,51 @@
         <is>
           <t>Mascarado ou Magma? qual é mais bonita? 👇
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #viralvideo #foryou #fyp #robloxbrasil #robloxedit #gamerbrasil #minigames #shorts</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #viralvideo #foryou #fyp #robloxbrasil #robloxedit #gamerbrasil #minigames #shorts</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="2" t="n">
+      <c r="B27" s="3" t="n">
         <v>75</v>
       </c>
-      <c r="C27" s="2" t="n">
+      <c r="C27" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>2026-10-20T12:30:00-03:00</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>videos/075_desafio_empilha.mp4</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/075_desafio_empilha.mp4</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I27" s="3" t="inlineStr">
         <is>
           <t>DESAFIO: faz 30 pontos no Empilha 😤 quem passar é lenda 👑 #shorts</t>
         </is>
@@ -1881,51 +1877,51 @@
         <is>
           <t>DESAFIO: faz 30 pontos no Empilha 😤 quem passar é lenda 👑
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #explore #fyp #foryou #robloxfyp #robloxgames #robloxbrasil #gamerbrasil #jogosonline #shorts</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #explore #fyp #foryou #robloxfyp #robloxgames #robloxbrasil #gamerbrasil #shorts</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B28" s="3" t="n">
         <v>74</v>
       </c>
-      <c r="C28" s="2" t="n">
+      <c r="C28" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr">
         <is>
           <t>2026-10-20T17:00:00-03:00</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>videos/074_tutorial_passos_7.mp4</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/074_tutorial_passos_7.mp4</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>como jogar em 3 passos 👇 passo fácil: entra no site 🔗 → pega um jogo rápido ⏱️ → #shorts</t>
         </is>
@@ -1934,51 +1930,51 @@
         <is>
           <t>como jogar em 3 passos 👇 passo fácil: entra no site 🔗 → pega um jogo rápido ⏱️ → vicia 🫠
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #viralvideo #viral #fyp #robloxedit #robloxfyp #jogosdecelular #jogosonline #shorts</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viralvideo #viral #fyp #robloxedit #robloxfyp #jogosdecelular #shorts</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B29" s="3" t="n">
         <v>73</v>
       </c>
-      <c r="C29" s="2" t="n">
+      <c r="C29" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>2026-10-20T20:30:00-03:00</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>videos/073_desafio_corte.mp4</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/073_desafio_corte.mp4</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="I29" s="3" t="inlineStr">
         <is>
           <t>DESAFIO: faz 10 pontos no Corte 😤 manda print nos comentários 📸 #shorts</t>
         </is>
@@ -1987,10 +1983,10 @@
         <is>
           <t>DESAFIO: faz 10 pontos no Corte 😤 manda print nos comentários 📸
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #viralvideo #trend #foryou #robloxbrasil #robloxfyp #roblox #minigames #jogosonline #shorts</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #viralvideo #trend #foryou #robloxbrasil #robloxfyp #minigames #shorts</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -2036,11 +2032,11 @@
           <t>eu às 22h: só uma partida / eu às 3h: 😭 #shorts</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>eu às 22h: só uma partida / eu às 3h: 😭
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #viral #fyp #explore #roblox #robloxgames #mobilegames #jogosdecelular #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #explore #robloxgames #mobilegames #jogosdecelular #shorts</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2089,11 +2085,11 @@
           <t>roda em celular fraco? roda leve no navegador 📱 #shorts</t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>roda em celular fraco? roda leve no navegador 📱
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #viral #foryou #paravoce #robloxedit #robloxfyp #robloxbrasil #gamerbrasil #mobilegames #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #fyp #viral #foryou #paravoce #robloxedit #robloxfyp #robloxbrasil #gamerbrasil #shorts</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2142,11 +2138,11 @@
           <t>skin do dia: Raio (Épico) ✨ #shorts</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>skin do dia: Raio (Épico) ✨
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #paravoce #trend #fyp #robloxfyp #roblox #jogosonline #jogosdecelular #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #paravoce #trend #fyp #robloxfyp #jogosdecelular #shorts</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2195,11 +2191,11 @@
           <t>DESAFIO: faz 20 pontos no Hélice 😤 duvido tu bater 😤 #shorts</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>DESAFIO: faz 20 pontos no Hélice 😤 duvido tu bater 😤
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #fyp #viral #explore #robloxbrasil #roblox #robloxfyp #jogosdecelular #jogosonline #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #fyp #viral #explore #robloxbrasil #robloxfyp #jogosdecelular #shorts</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2209,41 +2205,41 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B34" s="3" t="n">
         <v>68</v>
       </c>
-      <c r="C34" s="2" t="n">
+      <c r="C34" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>22/10/2026</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>2026-10-22T09:00:00-03:00</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>videos/068_tutorial_passos_2.mp4</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/068_tutorial_passos_2.mp4</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="I34" s="3" t="inlineStr">
         <is>
           <t>como jogar em 3 passos 👇 abre o navegador 🌐 → digita kavixbrasil.com.br ⌨️ → pro #shorts</t>
         </is>
@@ -2252,51 +2248,51 @@
         <is>
           <t>como jogar em 3 passos 👇 abre o navegador 🌐 → digita kavixbrasil.com.br ⌨️ → pronto, já tá jogando 🙌
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #fyp #paravoce #viral #robloxbrasil #robloxedit #mobilegames #minigames #shorts</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #fyp #paravoce #viral #robloxbrasil #robloxedit #mobilegames #minigames #shorts</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="2" t="n">
+      <c r="B35" s="3" t="n">
         <v>67</v>
       </c>
-      <c r="C35" s="2" t="n">
+      <c r="C35" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>22/10/2026</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>2026-10-22T12:30:00-03:00</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>videos/067_duelo_skins_aurora_vs_galaxia.mp4</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/067_duelo_skins_aurora_vs_galaxia.mp4</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="I35" s="3" t="inlineStr">
         <is>
           <t>Aurora ou Galáxia? qual é mais bonita? 👇 #shorts</t>
         </is>
@@ -2305,51 +2301,51 @@
         <is>
           <t>Aurora ou Galáxia? qual é mais bonita? 👇
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #viral #explore #fyp #robloxbrasil #roblox #robloxfyp #gamerbrasil #mobilegames #shorts</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #explore #fyp #robloxbrasil #robloxfyp #gamerbrasil #mobilegames #shorts</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="2" t="n">
+      <c r="B36" s="3" t="n">
         <v>66</v>
       </c>
-      <c r="C36" s="2" t="n">
+      <c r="C36" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>22/10/2026</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F36" s="3" t="inlineStr">
         <is>
           <t>2026-10-22T17:00:00-03:00</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G36" s="3" t="inlineStr">
         <is>
           <t>videos/066_tier_list_tier_list_dos_mais_satisfatorios.mp4</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H36" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/066_tier_list_tier_list_dos_mais_satisfatorios.mp4</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
+      <c r="I36" s="3" t="inlineStr">
         <is>
           <t>tier list dos mais satisfatórios 🔥 concorda? #shorts</t>
         </is>
@@ -2358,51 +2354,51 @@
         <is>
           <t>tier list dos mais satisfatórios 🔥 concorda?
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #paravoce #explore #viral #roblox #robloxgames #jogosdecelular #minigames #shorts</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #fyp #paravoce #explore #viral #robloxgames #jogosdecelular #minigames #shorts</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="2" t="n">
+      <c r="B37" s="3" t="n">
         <v>65</v>
       </c>
-      <c r="C37" s="2" t="n">
+      <c r="C37" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>22/10/2026</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>2026-10-22T20:30:00-03:00</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>videos/065_desafio_ponte.mp4</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/065_desafio_ponte.mp4</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="I37" s="3" t="inlineStr">
         <is>
           <t>DESAFIO: faz 30 pontos no Ponte 😤 quem passar é lenda 👑 #shorts</t>
         </is>
@@ -2411,10 +2407,10 @@
         <is>
           <t>DESAFIO: faz 30 pontos no Ponte 😤 quem passar é lenda 👑
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #explore #paravoce #foryou #robloxedit #robloxgames #roblox #gamerbrasil #jogosgratis #shorts</t>
-        </is>
-      </c>
-      <c r="K37" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #explore #paravoce #foryou #robloxedit #robloxgames #gamerbrasil #shorts</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -2460,11 +2456,11 @@
           <t>qual é o site? kavixbrasil.com.br 🔗 #shorts</t>
         </is>
       </c>
-      <c r="J38" s="4" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>qual é o site? kavixbrasil.com.br 🔗
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #paravoce #viral #trend #robloxgames #robloxfyp #jogosonline #jogosdecelular #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #fyp #paravoce #viral #trend #robloxgames #robloxfyp #jogosdecelular #shorts</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2513,11 +2509,11 @@
           <t>skin do dia: Cor Kavix (Épico) ✨ #shorts</t>
         </is>
       </c>
-      <c r="J39" s="4" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>skin do dia: Cor Kavix (Épico) ✨
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #foryou #fyp #trend #robloxedit #robloxfyp #robloxbrasil #minigames #gamerbrasil #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #foryou #fyp #trend #robloxedit #robloxfyp #robloxbrasil #minigames #shorts</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2566,11 +2562,11 @@
           <t>DESAFIO: faz 30 pontos no Sinal 😤 quem passar é lenda 👑 #shorts</t>
         </is>
       </c>
-      <c r="J40" s="4" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>DESAFIO: faz 30 pontos no Sinal 😤 quem passar é lenda 👑
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #explore #trend #viralvideo #robloxgames #robloxedit #jogosgratis #minigames #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #explore #trend #viralvideo #robloxgames #robloxedit #shorts</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2619,11 +2615,11 @@
           <t>meu recorde: 12 / meu irmão: 47 😭 #shorts</t>
         </is>
       </c>
-      <c r="J41" s="4" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>meu recorde: 12 / meu irmão: 47 😭
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #explore #trend #fyp #robloxfyp #robloxbrasil #robloxedit #gamerbrasil #jogosgratis #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #explore #trend #fyp #robloxfyp #robloxbrasil #robloxedit #shorts</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -2633,41 +2629,41 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="3" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="2" t="n">
+      <c r="B42" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="C42" s="2" t="n">
+      <c r="C42" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D42" s="3" t="inlineStr">
         <is>
           <t>24/10/2026</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E42" s="3" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F42" s="3" t="inlineStr">
         <is>
           <t>2026-10-24T09:00:00-03:00</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G42" s="3" t="inlineStr">
         <is>
           <t>videos/060_desafio_pega_tudo.mp4</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="H42" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/060_desafio_pega_tudo.mp4</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
+      <c r="I42" s="3" t="inlineStr">
         <is>
           <t>DESAFIO: faz 30 pontos no Pega Tudo 😤 quem passar é lenda 👑 #shorts</t>
         </is>
@@ -2676,51 +2672,51 @@
         <is>
           <t>DESAFIO: faz 30 pontos no Pega Tudo 😤 quem passar é lenda 👑
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #paravoce #viralvideo #viral #roblox #robloxbrasil #jogosonline #jogosdecelular #shorts</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #fyp #paravoce #viralvideo #viral #robloxbrasil #jogosdecelular #shorts</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="3" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="2" t="n">
+      <c r="B43" s="3" t="n">
         <v>59</v>
       </c>
-      <c r="C43" s="2" t="n">
+      <c r="C43" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>24/10/2026</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>2026-10-24T12:30:00-03:00</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>videos/059_pergunta_da_pra_jogar_no_pc.mp4</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/059_pergunta_da_pra_jogar_no_pc.mp4</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr">
+      <c r="I43" s="3" t="inlineStr">
         <is>
           <t>dá pra jogar no PC? dá sim, no navegador do PC 💻 #shorts</t>
         </is>
@@ -2729,51 +2725,51 @@
         <is>
           <t>dá pra jogar no PC? dá sim, no navegador do PC 💻
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #trend #viral #fyp #robloxedit #roblox #robloxgames #minigames #jogosdecelular #shorts</t>
-        </is>
-      </c>
-      <c r="K43" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #trend #viral #fyp #robloxedit #robloxgames #minigames #jogosdecelular #shorts</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="3" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="2" t="n">
+      <c r="B44" s="3" t="n">
         <v>58</v>
       </c>
-      <c r="C44" s="2" t="n">
+      <c r="C44" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
         <is>
           <t>24/10/2026</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E44" s="3" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F44" s="3" t="inlineStr">
         <is>
           <t>2026-10-24T17:00:00-03:00</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G44" s="3" t="inlineStr">
         <is>
           <t>videos/058_duelo_skins_cor_amizade_vs_bombeiro.mp4</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="H44" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/058_duelo_skins_cor_amizade_vs_bombeiro.mp4</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr">
+      <c r="I44" s="3" t="inlineStr">
         <is>
           <t>Cor Amizade ou Bombeiro? qual é mais bonita? 👇 #shorts</t>
         </is>
@@ -2782,51 +2778,51 @@
         <is>
           <t>Cor Amizade ou Bombeiro? qual é mais bonita? 👇
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #explore #viralvideo #paravoce #robloxfyp #robloxbrasil #gamerbrasil #mobilegames #shorts</t>
-        </is>
-      </c>
-      <c r="K44" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #explore #viralvideo #paravoce #robloxfyp #robloxbrasil #shorts</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="3" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="2" t="n">
+      <c r="B45" s="3" t="n">
         <v>57</v>
       </c>
-      <c r="C45" s="2" t="n">
+      <c r="C45" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>24/10/2026</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E45" s="3" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>2026-10-24T20:30:00-03:00</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>videos/057_tutorial_passos_6.mp4</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/057_tutorial_passos_6.mp4</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="I45" s="3" t="inlineStr">
         <is>
           <t>como jogar em 3 passos 👇 link na bio 🔗 → escolhe o jogo 🎮 → joga de graça 🎮 #shorts</t>
         </is>
@@ -2835,10 +2831,10 @@
         <is>
           <t>como jogar em 3 passos 👇 link na bio 🔗 → escolhe o jogo 🎮 → joga de graça 🎮
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #fyp #trend #paravoce #robloxgames #robloxfyp #robloxedit #jogosdecelular #jogosgratis #shorts</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #trend #paravoce #robloxgames #robloxfyp #robloxedit #shorts</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -2884,11 +2880,11 @@
           <t>tier list pra jogar no ônibus 🔥 concorda? #shorts</t>
         </is>
       </c>
-      <c r="J46" s="4" t="inlineStr">
+      <c r="J46" t="inlineStr">
         <is>
           <t>tier list pra jogar no ônibus 🔥 concorda?
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #viral #fyp #foryou #robloxbrasil #robloxfyp #jogosgratis #mobilegames #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #foryou #robloxbrasil #robloxfyp #jogosgratis #mobilegames #shorts</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -2937,11 +2933,11 @@
           <t>eu jurando que é o último / eu 10 jogos depois: 😭 #shorts</t>
         </is>
       </c>
-      <c r="J47" s="4" t="inlineStr">
+      <c r="J47" t="inlineStr">
         <is>
           <t>eu jurando que é o último / eu 10 jogos depois: 😭
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #viral #viralvideo #trend #robloxgames #roblox #robloxedit #minigames #jogosgratis #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #fyp #viral #viralvideo #trend #robloxgames #robloxedit #minigames #shorts</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -2990,11 +2986,11 @@
           <t>DESAFIO: faz 15 pontos no Pulso 😤 marca quem consegue 👇 #shorts</t>
         </is>
       </c>
-      <c r="J48" s="4" t="inlineStr">
+      <c r="J48" t="inlineStr">
         <is>
           <t>DESAFIO: faz 15 pontos no Pulso 😤 marca quem consegue 👇
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #trend #paravoce #viralvideo #roblox #robloxbrasil #minigames #mobilegames #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #trend #paravoce #viralvideo #robloxbrasil #minigames #shorts</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3043,11 +3039,11 @@
           <t>skin do dia: Astronauta (Lendário) ✨ #shorts</t>
         </is>
       </c>
-      <c r="J49" s="4" t="inlineStr">
+      <c r="J49" t="inlineStr">
         <is>
           <t>skin do dia: Astronauta (Lendário) ✨
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #foryou #paravoce #viral #robloxfyp #robloxgames #robloxbrasil #gamerbrasil #jogosgratis #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #fyp #foryou #paravoce #viral #robloxfyp #robloxgames #robloxbrasil #gamerbrasil #shorts</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3057,41 +3053,41 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="3" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="2" t="n">
+      <c r="B50" s="3" t="n">
         <v>52</v>
       </c>
-      <c r="C50" s="2" t="n">
+      <c r="C50" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>26/10/2026</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E50" s="3" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F50" s="3" t="inlineStr">
         <is>
           <t>2026-10-26T09:00:00-03:00</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G50" s="3" t="inlineStr">
         <is>
           <t>videos/052_desafio_espinhos.mp4</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="H50" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/052_desafio_espinhos.mp4</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr">
+      <c r="I50" s="3" t="inlineStr">
         <is>
           <t>DESAFIO: faz 10 pontos no Espinhos 😤 manda print nos comentários 📸 #shorts</t>
         </is>
@@ -3100,51 +3096,51 @@
         <is>
           <t>DESAFIO: faz 10 pontos no Espinhos 😤 manda print nos comentários 📸
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #fyp #viralvideo #foryou #robloxgames #roblox #jogosdecelular #jogosgratis #shorts</t>
-        </is>
-      </c>
-      <c r="K50" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #viralvideo #foryou #robloxgames #jogosdecelular #jogosgratis #shorts</t>
+        </is>
+      </c>
+      <c r="K50" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="2" t="n">
+      <c r="B51" s="3" t="n">
         <v>51</v>
       </c>
-      <c r="C51" s="2" t="n">
+      <c r="C51" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>26/10/2026</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>2026-10-26T12:30:00-03:00</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>videos/051_skin_do_dia_aura_cosmos.mp4</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/051_skin_do_dia_aura_cosmos.mp4</t>
         </is>
       </c>
-      <c r="I51" s="2" t="inlineStr">
+      <c r="I51" s="3" t="inlineStr">
         <is>
           <t>skin do dia: Aura Cosmos (Lendário) ✨ #shorts</t>
         </is>
@@ -3153,51 +3149,51 @@
         <is>
           <t>skin do dia: Aura Cosmos (Lendário) ✨
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #viral #trend #fyp #robloxfyp #robloxgames #roblox #gamerbrasil #mobilegames #shorts</t>
-        </is>
-      </c>
-      <c r="K51" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #trend #fyp #robloxfyp #robloxgames #gamerbrasil #mobilegames #shorts</t>
+        </is>
+      </c>
+      <c r="K51" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" s="3" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="2" t="n">
+      <c r="B52" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="C52" s="2" t="n">
+      <c r="C52" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
         <is>
           <t>26/10/2026</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E52" s="3" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F52" s="3" t="inlineStr">
         <is>
           <t>2026-10-26T17:00:00-03:00</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G52" s="3" t="inlineStr">
         <is>
           <t>videos/050_pergunta_tem_jogo_de_reflexo.mp4</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="H52" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/050_pergunta_tem_jogo_de_reflexo.mp4</t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr">
+      <c r="I52" s="3" t="inlineStr">
         <is>
           <t>tem jogo de reflexo? tem vários: Pulso, Sinal, Corte ⚡ #shorts</t>
         </is>
@@ -3206,51 +3202,51 @@
         <is>
           <t>tem jogo de reflexo? tem vários: Pulso, Sinal, Corte ⚡
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #paravoce #foryou #explore #robloxfyp #robloxgames #mobilegames #jogosonline #shorts</t>
-        </is>
-      </c>
-      <c r="K52" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #paravoce #foryou #explore #robloxfyp #robloxgames #mobilegames #shorts</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" s="3" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="2" t="n">
+      <c r="B53" s="3" t="n">
         <v>49</v>
       </c>
-      <c r="C53" s="2" t="n">
+      <c r="C53" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>26/10/2026</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E53" s="3" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>2026-10-26T20:30:00-03:00</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>videos/049_meme_mae.mp4</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="H53" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/049_meme_mae.mp4</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr">
+      <c r="I53" s="3" t="inlineStr">
         <is>
           <t>minha mãe: vai dormir / eu no KAVIX: 😭 #shorts</t>
         </is>
@@ -3259,10 +3255,10 @@
         <is>
           <t>minha mãe: vai dormir / eu no KAVIX: 😭
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #trend #foryou #explore #robloxfyp #robloxedit #roblox #mobilegames #gamerbrasil #shorts</t>
-        </is>
-      </c>
-      <c r="K53" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #trend #foryou #explore #robloxfyp #robloxedit #mobilegames #shorts</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -3308,11 +3304,11 @@
           <t>DESAFIO: faz 25 pontos no Balanço 😤 comenta teu recorde 👇 #shorts</t>
         </is>
       </c>
-      <c r="J54" s="4" t="inlineStr">
+      <c r="J54" t="inlineStr">
         <is>
           <t>DESAFIO: faz 25 pontos no Balanço 😤 comenta teu recorde 👇
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #foryou #explore #viralvideo #robloxbrasil #robloxgames #jogosonline #jogosdecelular #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #foryou #explore #viralvideo #robloxbrasil #robloxgames #jogosdecelular #shorts</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3361,11 +3357,11 @@
           <t>como jogar em 3 passos 👇 sem baixar nada 🙌 → toca no jogo 👆 → segura o recorde 🏆 #shorts</t>
         </is>
       </c>
-      <c r="J55" s="4" t="inlineStr">
+      <c r="J55" t="inlineStr">
         <is>
           <t>como jogar em 3 passos 👇 sem baixar nada 🙌 → toca no jogo 👆 → segura o recorde 🏆
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #paravoce #foryou #fyp #robloxgames #robloxfyp #robloxbrasil #gamerbrasil #minigames #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #paravoce #foryou #fyp #robloxgames #robloxfyp #robloxbrasil #gamerbrasil #shorts</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3414,11 +3410,11 @@
           <t>DESAFIO: faz 10 pontos no Bolhas 😤 manda print nos comentários 📸 #shorts</t>
         </is>
       </c>
-      <c r="J56" s="4" t="inlineStr">
+      <c r="J56" t="inlineStr">
         <is>
           <t>DESAFIO: faz 10 pontos no Bolhas 😤 manda print nos comentários 📸
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #explore #trend #viral #robloxfyp #robloxedit #jogosgratis #jogosdecelular #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #fyp #explore #trend #viral #robloxfyp #robloxedit #jogosgratis #shorts</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -3467,11 +3463,11 @@
           <t>segunda-feira / eu no ônibus jogando: 😭 #shorts</t>
         </is>
       </c>
-      <c r="J57" s="4" t="inlineStr">
+      <c r="J57" t="inlineStr">
         <is>
           <t>segunda-feira / eu no ônibus jogando: 😭
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #trend #paravoce #foryou #robloxfyp #robloxgames #roblox #mobilegames #jogosdecelular #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #trend #paravoce #foryou #robloxfyp #robloxgames #mobilegames #shorts</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -3481,41 +3477,41 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" s="3" t="n">
         <v>57</v>
       </c>
-      <c r="B58" s="2" t="n">
+      <c r="B58" s="3" t="n">
         <v>44</v>
       </c>
-      <c r="C58" s="2" t="n">
+      <c r="C58" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E58" s="3" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F58" s="3" t="inlineStr">
         <is>
           <t>2026-10-28T09:00:00-03:00</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G58" s="3" t="inlineStr">
         <is>
           <t>videos/044_pergunta_precisa_baixar_alguma_coisa.mp4</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="H58" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/044_pergunta_precisa_baixar_alguma_coisa.mp4</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr">
+      <c r="I58" s="3" t="inlineStr">
         <is>
           <t>precisa baixar alguma coisa? não! roda direto no navegador 🙌 #shorts</t>
         </is>
@@ -3524,51 +3520,51 @@
         <is>
           <t>precisa baixar alguma coisa? não! roda direto no navegador 🙌
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #trend #explore #paravoce #robloxgames #robloxbrasil #jogosonline #gamerbrasil #shorts</t>
-        </is>
-      </c>
-      <c r="K58" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #trend #explore #paravoce #robloxgames #robloxbrasil #shorts</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="3" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="2" t="n">
+      <c r="B59" s="3" t="n">
         <v>43</v>
       </c>
-      <c r="C59" s="2" t="n">
+      <c r="C59" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E59" s="3" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="F59" s="3" t="inlineStr">
         <is>
           <t>2026-10-28T12:30:00-03:00</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr">
+      <c r="G59" s="3" t="inlineStr">
         <is>
           <t>videos/043_duelo_skins_viseira_de_chama_vs_prisma.mp4</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="H59" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/043_duelo_skins_viseira_de_chama_vs_prisma.mp4</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr">
+      <c r="I59" s="3" t="inlineStr">
         <is>
           <t>Viseira de Chama ou Prisma? qual é mais bonita? 👇 #shorts</t>
         </is>
@@ -3577,51 +3573,51 @@
         <is>
           <t>Viseira de Chama ou Prisma? qual é mais bonita? 👇
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #foryou #trend #viralvideo #robloxgames #robloxedit #roblox #jogosdecelular #minigames #shorts</t>
-        </is>
-      </c>
-      <c r="K59" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #foryou #trend #viralvideo #robloxgames #robloxedit #jogosdecelular #shorts</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="3" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="2" t="n">
+      <c r="B60" s="3" t="n">
         <v>42</v>
       </c>
-      <c r="C60" s="2" t="n">
+      <c r="C60" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D60" s="3" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E60" s="3" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F60" s="3" t="inlineStr">
         <is>
           <t>2026-10-28T17:00:00-03:00</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>videos/042_desafio_encaixe.mp4</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="H60" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/042_desafio_encaixe.mp4</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr">
+      <c r="I60" s="3" t="inlineStr">
         <is>
           <t>DESAFIO: faz 15 pontos no Encaixe 😤 marca quem consegue 👇 #shorts</t>
         </is>
@@ -3630,51 +3626,51 @@
         <is>
           <t>DESAFIO: faz 15 pontos no Encaixe 😤 marca quem consegue 👇
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #foryou #viralvideo #trend #robloxgames #robloxfyp #jogosonline #mobilegames #shorts</t>
-        </is>
-      </c>
-      <c r="K60" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #foryou #viralvideo #trend #robloxgames #robloxfyp #mobilegames #shorts</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="3" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="2" t="n">
+      <c r="B61" s="3" t="n">
         <v>41</v>
       </c>
-      <c r="C61" s="2" t="n">
+      <c r="C61" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D61" s="3" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E61" s="3" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F61" s="3" t="inlineStr">
         <is>
           <t>2026-10-28T20:30:00-03:00</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G61" s="3" t="inlineStr">
         <is>
           <t>videos/041_skin_do_dia_mago.mp4</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="H61" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/041_skin_do_dia_mago.mp4</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr">
+      <c r="I61" s="3" t="inlineStr">
         <is>
           <t>skin do dia: Mago (Lendário) ✨ #shorts</t>
         </is>
@@ -3683,10 +3679,10 @@
         <is>
           <t>skin do dia: Mago (Lendário) ✨
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #viralvideo #viral #paravoce #robloxgames #robloxfyp #robloxbrasil #mobilegames #jogosgratis #shorts</t>
-        </is>
-      </c>
-      <c r="K61" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #fyp #viralvideo #viral #paravoce #robloxgames #robloxfyp #robloxbrasil #shorts</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -3732,11 +3728,11 @@
           <t>DESAFIO: faz 25 pontos no Boliche 😤 comenta teu recorde 👇 #shorts</t>
         </is>
       </c>
-      <c r="J62" s="4" t="inlineStr">
+      <c r="J62" t="inlineStr">
         <is>
           <t>DESAFIO: faz 25 pontos no Boliche 😤 comenta teu recorde 👇
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #foryou #fyp #paravoce #robloxbrasil #robloxedit #jogosonline #jogosgratis #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #foryou #fyp #paravoce #robloxbrasil #robloxedit #jogosgratis #shorts</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -3785,11 +3781,11 @@
           <t>skin do dia: Aura Sombria (Épico) ✨ #shorts</t>
         </is>
       </c>
-      <c r="J63" s="4" t="inlineStr">
+      <c r="J63" t="inlineStr">
         <is>
           <t>skin do dia: Aura Sombria (Épico) ✨
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #viral #paravoce #foryou #robloxedit #robloxfyp #robloxgames #minigames #jogosgratis #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #fyp #viral #paravoce #foryou #robloxedit #robloxfyp #robloxgames #minigames #shorts</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -3838,11 +3834,11 @@
           <t>qual o mais viciante? Empilha, fácil 🫠 #shorts</t>
         </is>
       </c>
-      <c r="J64" s="4" t="inlineStr">
+      <c r="J64" t="inlineStr">
         <is>
           <t>qual o mais viciante? Empilha, fácil 🫠
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #fyp #explore #viral #robloxbrasil #roblox #jogosonline #gamerbrasil #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #fyp #explore #viral #robloxbrasil #gamerbrasil #shorts</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -3891,11 +3887,11 @@
           <t>Viseira ou Cartola? qual é mais bonita? 👇 #shorts</t>
         </is>
       </c>
-      <c r="J65" s="4" t="inlineStr">
+      <c r="J65" t="inlineStr">
         <is>
           <t>Viseira ou Cartola? qual é mais bonita? 👇
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #explore #viralvideo #foryou #robloxfyp #roblox #robloxbrasil #jogosgratis #mobilegames #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #explore #viralvideo #foryou #robloxfyp #robloxbrasil #jogosgratis #shorts</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -3905,41 +3901,41 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="3" t="n">
         <v>65</v>
       </c>
-      <c r="B66" s="2" t="n">
+      <c r="B66" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="C66" s="2" t="n">
+      <c r="C66" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>30/10/2026</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E66" s="3" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F66" s="3" t="inlineStr">
         <is>
           <t>2026-10-30T09:00:00-03:00</t>
         </is>
       </c>
-      <c r="G66" s="2" t="inlineStr">
+      <c r="G66" s="3" t="inlineStr">
         <is>
           <t>videos/036_tutorial_passos_3.mp4</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr">
+      <c r="H66" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/036_tutorial_passos_3.mp4</t>
         </is>
       </c>
-      <c r="I66" s="2" t="inlineStr">
+      <c r="I66" s="3" t="inlineStr">
         <is>
           <t>como jogar em 3 passos 👇 no celular ou no PC 📱💻 → entra no site 🔗 → cria conta e #shorts</t>
         </is>
@@ -3948,51 +3944,51 @@
         <is>
           <t>como jogar em 3 passos 👇 no celular ou no PC 📱💻 → entra no site 🔗 → cria conta e ganha itens 🎁
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #viralvideo #trend #explore #robloxedit #robloxbrasil #jogosdecelular #jogosgratis #shorts</t>
-        </is>
-      </c>
-      <c r="K66" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #viralvideo #trend #explore #robloxedit #robloxbrasil #shorts</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" s="3" t="n">
         <v>66</v>
       </c>
-      <c r="B67" s="2" t="n">
+      <c r="B67" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="C67" s="2" t="n">
+      <c r="C67" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="D67" s="3" t="inlineStr">
         <is>
           <t>30/10/2026</t>
         </is>
       </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="E67" s="3" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F67" s="3" t="inlineStr">
         <is>
           <t>2026-10-30T12:30:00-03:00</t>
         </is>
       </c>
-      <c r="G67" s="2" t="inlineStr">
+      <c r="G67" s="3" t="inlineStr">
         <is>
           <t>videos/035_desafio_quebra_blocos.mp4</t>
         </is>
       </c>
-      <c r="H67" s="2" t="inlineStr">
+      <c r="H67" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/035_desafio_quebra_blocos.mp4</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr">
+      <c r="I67" s="3" t="inlineStr">
         <is>
           <t>DESAFIO: faz 20 pontos no Quebra Blocos 😤 duvido tu bater 😤 #shorts</t>
         </is>
@@ -4001,51 +3997,51 @@
         <is>
           <t>DESAFIO: faz 20 pontos no Quebra Blocos 😤 duvido tu bater 😤
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #foryou #explore #viral #robloxfyp #robloxedit #roblox #gamerbrasil #minigames #shorts</t>
-        </is>
-      </c>
-      <c r="K67" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #fyp #foryou #explore #viral #robloxfyp #robloxedit #gamerbrasil #minigames #shorts</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" s="3" t="n">
         <v>67</v>
       </c>
-      <c r="B68" s="2" t="n">
+      <c r="B68" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="C68" s="2" t="n">
+      <c r="C68" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="D68" s="3" t="inlineStr">
         <is>
           <t>30/10/2026</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E68" s="3" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="F68" s="3" t="inlineStr">
         <is>
           <t>2026-10-30T17:00:00-03:00</t>
         </is>
       </c>
-      <c r="G68" s="2" t="inlineStr">
+      <c r="G68" s="3" t="inlineStr">
         <is>
           <t>videos/034_meme_wifi.mp4</t>
         </is>
       </c>
-      <c r="H68" s="2" t="inlineStr">
+      <c r="H68" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/034_meme_wifi.mp4</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr">
+      <c r="I68" s="3" t="inlineStr">
         <is>
           <t>quando o wifi cai / o KAVIX no navegador: 😭 #shorts</t>
         </is>
@@ -4054,51 +4050,51 @@
         <is>
           <t>quando o wifi cai / o KAVIX no navegador: 😭
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #viral #fyp #explore #robloxfyp #roblox #mobilegames #gamerbrasil #shorts</t>
-        </is>
-      </c>
-      <c r="K68" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #explore #robloxfyp #mobilegames #gamerbrasil #shorts</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" s="3" t="n">
         <v>68</v>
       </c>
-      <c r="B69" s="2" t="n">
+      <c r="B69" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="C69" s="2" t="n">
+      <c r="C69" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="D69" s="3" t="inlineStr">
         <is>
           <t>30/10/2026</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E69" s="3" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F69" s="3" t="inlineStr">
         <is>
           <t>2026-10-30T20:30:00-03:00</t>
         </is>
       </c>
-      <c r="G69" s="2" t="inlineStr">
+      <c r="G69" s="3" t="inlineStr">
         <is>
           <t>videos/033_desafio_pula_corda.mp4</t>
         </is>
       </c>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="H69" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/033_desafio_pula_corda.mp4</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr">
+      <c r="I69" s="3" t="inlineStr">
         <is>
           <t>DESAFIO: faz 25 pontos no Pula Corda 😤 comenta teu recorde 👇 #shorts</t>
         </is>
@@ -4107,10 +4103,10 @@
         <is>
           <t>DESAFIO: faz 25 pontos no Pula Corda 😤 comenta teu recorde 👇
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #foryou #viral #paravoce #robloxedit #robloxbrasil #robloxgames #minigames #mobilegames #shorts</t>
-        </is>
-      </c>
-      <c r="K69" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #fyp #foryou #viral #paravoce #robloxedit #robloxbrasil #robloxgames #minigames #shorts</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -4156,11 +4152,11 @@
           <t>como eu ganho skins? cria tua conta e já ganha itens 🎁 #shorts</t>
         </is>
       </c>
-      <c r="J70" s="4" t="inlineStr">
+      <c r="J70" t="inlineStr">
         <is>
           <t>como eu ganho skins? cria tua conta e já ganha itens 🎁
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #trend #paravoce #fyp #robloxgames #robloxfyp #jogosdecelular #jogosonline #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #trend #paravoce #fyp #robloxgames #robloxfyp #jogosdecelular #shorts</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4209,11 +4205,11 @@
           <t>meu amigo: esse é fácil / o nível 3: 😭 #shorts</t>
         </is>
       </c>
-      <c r="J71" s="4" t="inlineStr">
+      <c r="J71" t="inlineStr">
         <is>
           <t>meu amigo: esse é fácil / o nível 3: 😭
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #trend #viralvideo #foryou #robloxgames #robloxfyp #roblox #jogosonline #jogosgratis #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #trend #viralvideo #foryou #robloxgames #robloxfyp #jogosgratis #shorts</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4262,11 +4258,11 @@
           <t>skin do dia: Capacete Espacial (Épico) ✨ #shorts</t>
         </is>
       </c>
-      <c r="J72" s="4" t="inlineStr">
+      <c r="J72" t="inlineStr">
         <is>
           <t>skin do dia: Capacete Espacial (Épico) ✨
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #foryou #paravoce #viralvideo #robloxfyp #roblox #jogosonline #gamerbrasil #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #foryou #paravoce #viralvideo #robloxfyp #gamerbrasil #shorts</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -4315,11 +4311,11 @@
           <t>DESAFIO: faz 25 pontos no Fio 😤 comenta teu recorde 👇 #shorts</t>
         </is>
       </c>
-      <c r="J73" s="4" t="inlineStr">
+      <c r="J73" t="inlineStr">
         <is>
           <t>DESAFIO: faz 25 pontos no Fio 😤 comenta teu recorde 👇
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #paravoce #trend #viralvideo #robloxedit #robloxgames #robloxfyp #mobilegames #minigames #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #paravoce #trend #viralvideo #robloxedit #robloxgames #shorts</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -4329,41 +4325,41 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
+      <c r="A74" s="3" t="n">
         <v>73</v>
       </c>
-      <c r="B74" s="2" t="n">
+      <c r="B74" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="C74" s="2" t="n">
+      <c r="C74" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="D74" s="2" t="inlineStr">
+      <c r="D74" s="3" t="inlineStr">
         <is>
           <t>01/11/2026</t>
         </is>
       </c>
-      <c r="E74" s="2" t="inlineStr">
+      <c r="E74" s="3" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr">
+      <c r="F74" s="3" t="inlineStr">
         <is>
           <t>2026-11-01T09:00:00-03:00</t>
         </is>
       </c>
-      <c r="G74" s="2" t="inlineStr">
+      <c r="G74" s="3" t="inlineStr">
         <is>
           <t>videos/028_tutorial_passos_10.mp4</t>
         </is>
       </c>
-      <c r="H74" s="2" t="inlineStr">
+      <c r="H74" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/028_tutorial_passos_10.mp4</t>
         </is>
       </c>
-      <c r="I74" s="2" t="inlineStr">
+      <c r="I74" s="3" t="inlineStr">
         <is>
           <t>como jogar em 3 passos 👇 chama teu amigo 👥 → cada um no seu celular 📱 → quem fiz #shorts</t>
         </is>
@@ -4372,51 +4368,51 @@
         <is>
           <t>como jogar em 3 passos 👇 chama teu amigo 👥 → cada um no seu celular 📱 → quem fizer mais ganha 🏆
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #paravoce #explore #foryou #roblox #robloxgames #jogosdecelular #mobilegames #shorts</t>
-        </is>
-      </c>
-      <c r="K74" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #paravoce #explore #foryou #robloxgames #jogosdecelular #mobilegames #shorts</t>
+        </is>
+      </c>
+      <c r="K74" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
+      <c r="A75" s="3" t="n">
         <v>74</v>
       </c>
-      <c r="B75" s="2" t="n">
+      <c r="B75" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="C75" s="2" t="n">
+      <c r="C75" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="D75" s="2" t="inlineStr">
+      <c r="D75" s="3" t="inlineStr">
         <is>
           <t>01/11/2026</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr">
+      <c r="E75" s="3" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="F75" s="2" t="inlineStr">
+      <c r="F75" s="3" t="inlineStr">
         <is>
           <t>2026-11-01T12:30:00-03:00</t>
         </is>
       </c>
-      <c r="G75" s="2" t="inlineStr">
+      <c r="G75" s="3" t="inlineStr">
         <is>
           <t>videos/027_tier_list_tier_list_de_reflexo.mp4</t>
         </is>
       </c>
-      <c r="H75" s="2" t="inlineStr">
+      <c r="H75" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/027_tier_list_tier_list_de_reflexo.mp4</t>
         </is>
       </c>
-      <c r="I75" s="2" t="inlineStr">
+      <c r="I75" s="3" t="inlineStr">
         <is>
           <t>tier list de reflexo 🔥 concorda? #shorts</t>
         </is>
@@ -4425,51 +4421,51 @@
         <is>
           <t>tier list de reflexo 🔥 concorda?
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #foryou #explore #paravoce #roblox #robloxgames #robloxbrasil #jogosonline #jogosdecelular #shorts</t>
-        </is>
-      </c>
-      <c r="K75" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #foryou #explore #paravoce #robloxgames #robloxbrasil #jogosdecelular #shorts</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="3" t="n">
         <v>75</v>
       </c>
-      <c r="B76" s="2" t="n">
+      <c r="B76" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="C76" s="2" t="n">
+      <c r="C76" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="D76" s="2" t="inlineStr">
+      <c r="D76" s="3" t="inlineStr">
         <is>
           <t>01/11/2026</t>
         </is>
       </c>
-      <c r="E76" s="2" t="inlineStr">
+      <c r="E76" s="3" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F76" s="2" t="inlineStr">
+      <c r="F76" s="3" t="inlineStr">
         <is>
           <t>2026-11-01T17:00:00-03:00</t>
         </is>
       </c>
-      <c r="G76" s="2" t="inlineStr">
+      <c r="G76" s="3" t="inlineStr">
         <is>
           <t>videos/026_desafio_zigue_zague.mp4</t>
         </is>
       </c>
-      <c r="H76" s="2" t="inlineStr">
+      <c r="H76" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/026_desafio_zigue_zague.mp4</t>
         </is>
       </c>
-      <c r="I76" s="2" t="inlineStr">
+      <c r="I76" s="3" t="inlineStr">
         <is>
           <t>DESAFIO: faz 30 pontos no Zigue-Zague 😤 quem passar é lenda 👑 #shorts</t>
         </is>
@@ -4478,51 +4474,51 @@
         <is>
           <t>DESAFIO: faz 30 pontos no Zigue-Zague 😤 quem passar é lenda 👑
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #foryou #viralvideo #trend #robloxfyp #robloxbrasil #jogosgratis #mobilegames #shorts</t>
-        </is>
-      </c>
-      <c r="K76" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #foryou #viralvideo #trend #robloxfyp #robloxbrasil #jogosgratis #shorts</t>
+        </is>
+      </c>
+      <c r="K76" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
+      <c r="A77" s="3" t="n">
         <v>76</v>
       </c>
-      <c r="B77" s="2" t="n">
+      <c r="B77" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="C77" s="2" t="n">
+      <c r="C77" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="D77" s="3" t="inlineStr">
         <is>
           <t>01/11/2026</t>
         </is>
       </c>
-      <c r="E77" s="2" t="inlineStr">
+      <c r="E77" s="3" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr">
+      <c r="F77" s="3" t="inlineStr">
         <is>
           <t>2026-11-01T20:30:00-03:00</t>
         </is>
       </c>
-      <c r="G77" s="2" t="inlineStr">
+      <c r="G77" s="3" t="inlineStr">
         <is>
           <t>videos/025_meme_real.mp4</t>
         </is>
       </c>
-      <c r="H77" s="2" t="inlineStr">
+      <c r="H77" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/025_meme_real.mp4</t>
         </is>
       </c>
-      <c r="I77" s="2" t="inlineStr">
+      <c r="I77" s="3" t="inlineStr">
         <is>
           <t>expectativa: jogo fácil ❌ / realidade: 😭 #shorts</t>
         </is>
@@ -4531,10 +4527,10 @@
         <is>
           <t>expectativa: jogo fácil ❌ / realidade: 😭
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #viral #fyp #viralvideo #robloxbrasil #robloxedit #robloxfyp #jogosgratis #jogosdecelular #shorts</t>
-        </is>
-      </c>
-      <c r="K77" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #viralvideo #robloxbrasil #robloxedit #robloxfyp #jogosgratis #shorts</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -4580,11 +4576,11 @@
           <t>Blindado ou Aura de Gelo? qual é mais bonita? 👇 #shorts</t>
         </is>
       </c>
-      <c r="J78" s="4" t="inlineStr">
+      <c r="J78" t="inlineStr">
         <is>
           <t>Blindado ou Aura de Gelo? qual é mais bonita? 👇
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #fyp #explore #viral #roblox #robloxedit #jogosgratis #mobilegames #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #fyp #explore #viral #robloxedit #jogosgratis #mobilegames #shorts</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -4633,11 +4629,11 @@
           <t>skin do dia: Aura Estelar (Lendário) ✨ #shorts</t>
         </is>
       </c>
-      <c r="J79" s="4" t="inlineStr">
+      <c r="J79" t="inlineStr">
         <is>
           <t>skin do dia: Aura Estelar (Lendário) ✨
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #explore #fyp #viralvideo #robloxgames #robloxfyp #robloxedit #jogosonline #jogosgratis #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #explore #fyp #viralvideo #robloxgames #robloxfyp #robloxedit #shorts</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -4686,11 +4682,11 @@
           <t>DESAFIO: faz 15 pontos no Passagem 😤 marca quem consegue 👇 #shorts</t>
         </is>
       </c>
-      <c r="J80" s="4" t="inlineStr">
+      <c r="J80" t="inlineStr">
         <is>
           <t>DESAFIO: faz 15 pontos no Passagem 😤 marca quem consegue 👇
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #viral #foryou #trend #robloxbrasil #roblox #jogosgratis #jogosdecelular #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #fyp #viral #foryou #trend #robloxbrasil #jogosgratis #jogosdecelular #shorts</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -4739,11 +4735,11 @@
           <t>dá pra jogar no intervalo? partidas rapidinhas ⏱️ #shorts</t>
         </is>
       </c>
-      <c r="J81" s="4" t="inlineStr">
+      <c r="J81" t="inlineStr">
         <is>
           <t>dá pra jogar no intervalo? partidas rapidinhas ⏱️
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #fyp #viral #paravoce #robloxedit #robloxgames #robloxfyp #jogosonline #jogosdecelular #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #fyp #viral #paravoce #robloxedit #robloxgames #robloxfyp #jogosdecelular #shorts</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -4753,41 +4749,41 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="3" t="n">
         <v>81</v>
       </c>
-      <c r="B82" s="2" t="n">
+      <c r="B82" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="C82" s="2" t="n">
+      <c r="C82" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="D82" s="2" t="inlineStr">
+      <c r="D82" s="3" t="inlineStr">
         <is>
           <t>03/11/2026</t>
         </is>
       </c>
-      <c r="E82" s="2" t="inlineStr">
+      <c r="E82" s="3" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F82" s="2" t="inlineStr">
+      <c r="F82" s="3" t="inlineStr">
         <is>
           <t>2026-11-03T09:00:00-03:00</t>
         </is>
       </c>
-      <c r="G82" s="2" t="inlineStr">
+      <c r="G82" s="3" t="inlineStr">
         <is>
           <t>videos/020_desafio_canhao.mp4</t>
         </is>
       </c>
-      <c r="H82" s="2" t="inlineStr">
+      <c r="H82" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/020_desafio_canhao.mp4</t>
         </is>
       </c>
-      <c r="I82" s="2" t="inlineStr">
+      <c r="I82" s="3" t="inlineStr">
         <is>
           <t>DESAFIO: faz 20 pontos no Canhão 😤 duvido tu bater 😤 #shorts</t>
         </is>
@@ -4796,51 +4792,51 @@
         <is>
           <t>DESAFIO: faz 20 pontos no Canhão 😤 duvido tu bater 😤
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #explore #foryou #fyp #robloxfyp #robloxbrasil #minigames #mobilegames #shorts</t>
-        </is>
-      </c>
-      <c r="K82" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #explore #foryou #fyp #robloxfyp #robloxbrasil #minigames #mobilegames #shorts</t>
+        </is>
+      </c>
+      <c r="K82" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
+      <c r="A83" s="3" t="n">
         <v>82</v>
       </c>
-      <c r="B83" s="2" t="n">
+      <c r="B83" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="C83" s="2" t="n">
+      <c r="C83" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="D83" s="2" t="inlineStr">
+      <c r="D83" s="3" t="inlineStr">
         <is>
           <t>03/11/2026</t>
         </is>
       </c>
-      <c r="E83" s="2" t="inlineStr">
+      <c r="E83" s="3" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="F83" s="2" t="inlineStr">
+      <c r="F83" s="3" t="inlineStr">
         <is>
           <t>2026-11-03T12:30:00-03:00</t>
         </is>
       </c>
-      <c r="G83" s="2" t="inlineStr">
+      <c r="G83" s="3" t="inlineStr">
         <is>
           <t>videos/019_meme_fio.mp4</t>
         </is>
       </c>
-      <c r="H83" s="2" t="inlineStr">
+      <c r="H83" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/019_meme_fio.mp4</t>
         </is>
       </c>
-      <c r="I83" s="2" t="inlineStr">
+      <c r="I83" s="3" t="inlineStr">
         <is>
           <t>eu achando que sou bom / o jogo Fio: 😭 #shorts</t>
         </is>
@@ -4849,51 +4845,51 @@
         <is>
           <t>eu achando que sou bom / o jogo Fio: 😭
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #paravoce #fyp #viral #robloxfyp #robloxbrasil #robloxgames #jogosgratis #jogosonline #shorts</t>
-        </is>
-      </c>
-      <c r="K83" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #paravoce #fyp #viral #robloxfyp #robloxbrasil #robloxgames #jogosgratis #shorts</t>
+        </is>
+      </c>
+      <c r="K83" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="3" t="n">
         <v>83</v>
       </c>
-      <c r="B84" s="2" t="n">
+      <c r="B84" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="C84" s="2" t="n">
+      <c r="C84" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="D84" s="2" t="inlineStr">
+      <c r="D84" s="3" t="inlineStr">
         <is>
           <t>03/11/2026</t>
         </is>
       </c>
-      <c r="E84" s="2" t="inlineStr">
+      <c r="E84" s="3" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F84" s="2" t="inlineStr">
+      <c r="F84" s="3" t="inlineStr">
         <is>
           <t>2026-11-03T17:00:00-03:00</t>
         </is>
       </c>
-      <c r="G84" s="2" t="inlineStr">
+      <c r="G84" s="3" t="inlineStr">
         <is>
           <t>videos/018_pergunta_tem_coisa_pra_quem_curte_roblox.mp4</t>
         </is>
       </c>
-      <c r="H84" s="2" t="inlineStr">
+      <c r="H84" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/018_pergunta_tem_coisa_pra_quem_curte_roblox.mp4</t>
         </is>
       </c>
-      <c r="I84" s="2" t="inlineStr">
+      <c r="I84" s="3" t="inlineStr">
         <is>
           <t>tem coisa pra quem curte Roblox? minigames rápidos e skins 👀 #shorts</t>
         </is>
@@ -4902,51 +4898,51 @@
         <is>
           <t>tem coisa pra quem curte Roblox? minigames rápidos e skins 👀
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #foryou #paravoce #explore #robloxfyp #roblox #minigames #gamerbrasil #shorts</t>
-        </is>
-      </c>
-      <c r="K84" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #foryou #paravoce #explore #robloxfyp #minigames #gamerbrasil #shorts</t>
+        </is>
+      </c>
+      <c r="K84" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
+      <c r="A85" s="3" t="n">
         <v>84</v>
       </c>
-      <c r="B85" s="2" t="n">
+      <c r="B85" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="C85" s="2" t="n">
+      <c r="C85" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="D85" s="2" t="inlineStr">
+      <c r="D85" s="3" t="inlineStr">
         <is>
           <t>03/11/2026</t>
         </is>
       </c>
-      <c r="E85" s="2" t="inlineStr">
+      <c r="E85" s="3" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="F85" s="2" t="inlineStr">
+      <c r="F85" s="3" t="inlineStr">
         <is>
           <t>2026-11-03T20:30:00-03:00</t>
         </is>
       </c>
-      <c r="G85" s="2" t="inlineStr">
+      <c r="G85" s="3" t="inlineStr">
         <is>
           <t>videos/017_skin_do_dia_aura_eletrica.mp4</t>
         </is>
       </c>
-      <c r="H85" s="2" t="inlineStr">
+      <c r="H85" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/017_skin_do_dia_aura_eletrica.mp4</t>
         </is>
       </c>
-      <c r="I85" s="2" t="inlineStr">
+      <c r="I85" s="3" t="inlineStr">
         <is>
           <t>skin do dia: Aura Elétrica (Épico) ✨ #shorts</t>
         </is>
@@ -4955,10 +4951,10 @@
         <is>
           <t>skin do dia: Aura Elétrica (Épico) ✨
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #explore #viralvideo #viral #robloxedit #robloxbrasil #roblox #jogosdecelular #jogosgratis #shorts</t>
-        </is>
-      </c>
-      <c r="K85" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #fyp #explore #viralvideo #viral #robloxedit #robloxbrasil #jogosdecelular #shorts</t>
+        </is>
+      </c>
+      <c r="K85" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -5004,11 +5000,11 @@
           <t>DESAFIO: faz 10 pontos no Órbita 😤 manda print nos comentários 📸 #shorts</t>
         </is>
       </c>
-      <c r="J86" s="4" t="inlineStr">
+      <c r="J86" t="inlineStr">
         <is>
           <t>DESAFIO: faz 10 pontos no Órbita 😤 manda print nos comentários 📸
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #paravoce #viral #explore #robloxedit #robloxbrasil #mobilegames #jogosonline #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #fyp #paravoce #viral #explore #robloxedit #robloxbrasil #mobilegames #shorts</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5057,11 +5053,11 @@
           <t>como jogar em 3 passos 👇 entra em kavixbrasil.com.br 🔗 → escolhe um dos 30 jogos #shorts</t>
         </is>
       </c>
-      <c r="J87" s="4" t="inlineStr">
+      <c r="J87" t="inlineStr">
         <is>
           <t>como jogar em 3 passos 👇 entra em kavixbrasil.com.br 🔗 → escolhe um dos 30 jogos 🎮 → joga e bate teu recorde 🔥
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #trend #fyp #foryou #roblox #robloxedit #robloxfyp #jogosonline #minigames #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #trend #fyp #foryou #robloxedit #robloxfyp #minigames #shorts</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -5110,11 +5106,11 @@
           <t>Faraó ou Coroa de Gelo? qual é mais bonita? 👇 #shorts</t>
         </is>
       </c>
-      <c r="J88" s="4" t="inlineStr">
+      <c r="J88" t="inlineStr">
         <is>
           <t>Faraó ou Coroa de Gelo? qual é mais bonita? 👇
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #foryou #trend #paravoce #robloxedit #robloxbrasil #gamerbrasil #mobilegames #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #foryou #trend #paravoce #robloxedit #robloxbrasil #gamerbrasil #shorts</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -5163,11 +5159,11 @@
           <t>skin do dia: Vulto (Épico) ✨ #shorts</t>
         </is>
       </c>
-      <c r="J89" s="4" t="inlineStr">
+      <c r="J89" t="inlineStr">
         <is>
           <t>skin do dia: Vulto (Épico) ✨
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #viralvideo #foryou #trend #robloxgames #robloxfyp #roblox #jogosgratis #jogosonline #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #viralvideo #foryou #trend #robloxgames #robloxfyp #jogosgratis #shorts</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -5177,41 +5173,41 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
+      <c r="A90" s="3" t="n">
         <v>89</v>
       </c>
-      <c r="B90" s="2" t="n">
+      <c r="B90" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="C90" s="2" t="n">
+      <c r="C90" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="D90" s="2" t="inlineStr">
+      <c r="D90" s="3" t="inlineStr">
         <is>
           <t>05/11/2026</t>
         </is>
       </c>
-      <c r="E90" s="2" t="inlineStr">
+      <c r="E90" s="3" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F90" s="2" t="inlineStr">
+      <c r="F90" s="3" t="inlineStr">
         <is>
           <t>2026-11-05T09:00:00-03:00</t>
         </is>
       </c>
-      <c r="G90" s="2" t="inlineStr">
+      <c r="G90" s="3" t="inlineStr">
         <is>
           <t>videos/012_pergunta_quantos_jogos_tem.mp4</t>
         </is>
       </c>
-      <c r="H90" s="2" t="inlineStr">
+      <c r="H90" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/012_pergunta_quantos_jogos_tem.mp4</t>
         </is>
       </c>
-      <c r="I90" s="2" t="inlineStr">
+      <c r="I90" s="3" t="inlineStr">
         <is>
           <t>quantos jogos tem? 30 jogos e contando 🔥 #shorts</t>
         </is>
@@ -5220,51 +5216,51 @@
         <is>
           <t>quantos jogos tem? 30 jogos e contando 🔥
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #foryou #trend #explore #robloxgames #robloxedit #jogosgratis #minigames #shorts</t>
-        </is>
-      </c>
-      <c r="K90" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #foryou #trend #explore #robloxgames #robloxedit #jogosgratis #shorts</t>
+        </is>
+      </c>
+      <c r="K90" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n">
+      <c r="A91" s="3" t="n">
         <v>90</v>
       </c>
-      <c r="B91" s="2" t="n">
+      <c r="B91" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="C91" s="2" t="n">
+      <c r="C91" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="D91" s="2" t="inlineStr">
+      <c r="D91" s="3" t="inlineStr">
         <is>
           <t>05/11/2026</t>
         </is>
       </c>
-      <c r="E91" s="2" t="inlineStr">
+      <c r="E91" s="3" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="F91" s="2" t="inlineStr">
+      <c r="F91" s="3" t="inlineStr">
         <is>
           <t>2026-11-05T12:30:00-03:00</t>
         </is>
       </c>
-      <c r="G91" s="2" t="inlineStr">
+      <c r="G91" s="3" t="inlineStr">
         <is>
           <t>videos/011_desafio_ricochete.mp4</t>
         </is>
       </c>
-      <c r="H91" s="2" t="inlineStr">
+      <c r="H91" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/011_desafio_ricochete.mp4</t>
         </is>
       </c>
-      <c r="I91" s="2" t="inlineStr">
+      <c r="I91" s="3" t="inlineStr">
         <is>
           <t>DESAFIO: faz 20 pontos no Ricochete 😤 duvido tu bater 😤 #shorts</t>
         </is>
@@ -5273,51 +5269,51 @@
         <is>
           <t>DESAFIO: faz 20 pontos no Ricochete 😤 duvido tu bater 😤
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #explore #trend #foryou #robloxedit #robloxgames #robloxfyp #jogosgratis #jogosonline #shorts</t>
-        </is>
-      </c>
-      <c r="K91" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #explore #trend #foryou #robloxedit #robloxgames #robloxfyp #shorts</t>
+        </is>
+      </c>
+      <c r="K91" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n">
+      <c r="A92" s="3" t="n">
         <v>91</v>
       </c>
-      <c r="B92" s="2" t="n">
+      <c r="B92" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="C92" s="2" t="n">
+      <c r="C92" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="D92" s="2" t="inlineStr">
+      <c r="D92" s="3" t="inlineStr">
         <is>
           <t>05/11/2026</t>
         </is>
       </c>
-      <c r="E92" s="2" t="inlineStr">
+      <c r="E92" s="3" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F92" s="2" t="inlineStr">
+      <c r="F92" s="3" t="inlineStr">
         <is>
           <t>2026-11-05T17:00:00-03:00</t>
         </is>
       </c>
-      <c r="G92" s="2" t="inlineStr">
+      <c r="G92" s="3" t="inlineStr">
         <is>
           <t>videos/010_meme_aula.mp4</t>
         </is>
       </c>
-      <c r="H92" s="2" t="inlineStr">
+      <c r="H92" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/010_meme_aula.mp4</t>
         </is>
       </c>
-      <c r="I92" s="2" t="inlineStr">
+      <c r="I92" s="3" t="inlineStr">
         <is>
           <t>o professor explicando / eu no intervalo: 😭 #shorts</t>
         </is>
@@ -5326,51 +5322,51 @@
         <is>
           <t>o professor explicando / eu no intervalo: 😭
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #fyp #viral #trend #robloxfyp #roblox #gamerbrasil #jogosgratis #shorts</t>
-        </is>
-      </c>
-      <c r="K92" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #fyp #viral #trend #robloxfyp #gamerbrasil #jogosgratis #shorts</t>
+        </is>
+      </c>
+      <c r="K92" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n">
+      <c r="A93" s="3" t="n">
         <v>92</v>
       </c>
-      <c r="B93" s="2" t="n">
+      <c r="B93" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="C93" s="2" t="n">
+      <c r="C93" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="D93" s="2" t="inlineStr">
+      <c r="D93" s="3" t="inlineStr">
         <is>
           <t>05/11/2026</t>
         </is>
       </c>
-      <c r="E93" s="2" t="inlineStr">
+      <c r="E93" s="3" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="F93" s="2" t="inlineStr">
+      <c r="F93" s="3" t="inlineStr">
         <is>
           <t>2026-11-05T20:30:00-03:00</t>
         </is>
       </c>
-      <c r="G93" s="2" t="inlineStr">
+      <c r="G93" s="3" t="inlineStr">
         <is>
           <t>videos/009_desafio_trampolim.mp4</t>
         </is>
       </c>
-      <c r="H93" s="2" t="inlineStr">
+      <c r="H93" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/009_desafio_trampolim.mp4</t>
         </is>
       </c>
-      <c r="I93" s="2" t="inlineStr">
+      <c r="I93" s="3" t="inlineStr">
         <is>
           <t>DESAFIO: faz 20 pontos no Trampolim 😤 duvido tu bater 😤 #shorts</t>
         </is>
@@ -5379,10 +5375,10 @@
         <is>
           <t>DESAFIO: faz 20 pontos no Trampolim 😤 duvido tu bater 😤
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #foryou #viral #paravoce #robloxbrasil #robloxfyp #robloxedit #mobilegames #jogosgratis #shorts</t>
-        </is>
-      </c>
-      <c r="K93" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #fyp #foryou #viral #paravoce #robloxbrasil #robloxfyp #robloxedit #mobilegames #shorts</t>
+        </is>
+      </c>
+      <c r="K93" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
@@ -5428,11 +5424,11 @@
           <t>tier list dos mais viciantes 🔥 concorda? #shorts</t>
         </is>
       </c>
-      <c r="J94" s="4" t="inlineStr">
+      <c r="J94" t="inlineStr">
         <is>
           <t>tier list dos mais viciantes 🔥 concorda?
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #explore #paravoce #trend #robloxfyp #robloxedit #jogosdecelular #minigames #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #explore #paravoce #trend #robloxfyp #robloxedit #shorts</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -5481,11 +5477,11 @@
           <t>como jogar em 3 passos 👇 cria tua conta 📝 → veste tua bolinha 👕 → desafia teus a #shorts</t>
         </is>
       </c>
-      <c r="J95" s="4" t="inlineStr">
+      <c r="J95" t="inlineStr">
         <is>
           <t>como jogar em 3 passos 👇 cria tua conta 📝 → veste tua bolinha 👕 → desafia teus amigos 😤
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #foryou #fyp #viral #robloxbrasil #robloxedit #roblox #jogosgratis #minigames #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #fyp #viral #robloxbrasil #robloxedit #jogosgratis #minigames #shorts</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -5534,11 +5530,11 @@
           <t>Coroa ou Óculos Espelhados? qual é mais bonita? 👇 #shorts</t>
         </is>
       </c>
-      <c r="J96" s="4" t="inlineStr">
+      <c r="J96" t="inlineStr">
         <is>
           <t>Coroa ou Óculos Espelhados? qual é mais bonita? 👇
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #fyp #paravoce #foryou #robloxbrasil #roblox #jogosgratis #jogosonline #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #paravoce #foryou #robloxbrasil #jogosgratis #shorts</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -5587,11 +5583,11 @@
           <t>DESAFIO: faz 15 pontos no Memória 😤 marca quem consegue 👇 #shorts</t>
         </is>
       </c>
-      <c r="J97" s="4" t="inlineStr">
+      <c r="J97" t="inlineStr">
         <is>
           <t>DESAFIO: faz 15 pontos no Memória 😤 marca quem consegue 👇
 Joga agora 👉 kavixbrasil.com.br (link na bio)
-#kavix #kavixarcade #foryou #paravoce #fyp #robloxedit #roblox #robloxgames #jogosonline #gamerbrasil #shorts</t>
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #foryou #paravoce #fyp #robloxedit #robloxgames #gamerbrasil #shorts</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -5601,41 +5597,41 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n">
+      <c r="A98" s="3" t="n">
         <v>97</v>
       </c>
-      <c r="B98" s="2" t="n">
+      <c r="B98" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="C98" s="2" t="n">
+      <c r="C98" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="D98" s="2" t="inlineStr">
+      <c r="D98" s="3" t="inlineStr">
         <is>
           <t>07/11/2026</t>
         </is>
       </c>
-      <c r="E98" s="2" t="inlineStr">
+      <c r="E98" s="3" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F98" s="2" t="inlineStr">
+      <c r="F98" s="3" t="inlineStr">
         <is>
           <t>2026-11-07T09:00:00-03:00</t>
         </is>
       </c>
-      <c r="G98" s="2" t="inlineStr">
+      <c r="G98" s="3" t="inlineStr">
         <is>
           <t>videos/004_pergunta_funciona_no_celular.mp4</t>
         </is>
       </c>
-      <c r="H98" s="2" t="inlineStr">
+      <c r="H98" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/004_pergunta_funciona_no_celular.mp4</t>
         </is>
       </c>
-      <c r="I98" s="2" t="inlineStr">
+      <c r="I98" s="3" t="inlineStr">
         <is>
           <t>funciona no celular? funciona! é só abrir o site 📱 #shorts</t>
         </is>
@@ -5644,51 +5640,51 @@
         <is>
           <t>funciona no celular? funciona! é só abrir o site 📱
 Salva esse vídeo e joga depois 📌 kavixbrasil.com.br
-#kavix #kavixarcade #paravoce #viralvideo #trend #roblox #robloxedit #jogosgratis #jogosonline #shorts</t>
-        </is>
-      </c>
-      <c r="K98" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #fyp #paravoce #viralvideo #trend #robloxedit #jogosgratis #shorts</t>
+        </is>
+      </c>
+      <c r="K98" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n">
+      <c r="A99" s="3" t="n">
         <v>98</v>
       </c>
-      <c r="B99" s="2" t="n">
+      <c r="B99" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C99" s="2" t="n">
+      <c r="C99" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="D99" s="2" t="inlineStr">
+      <c r="D99" s="3" t="inlineStr">
         <is>
           <t>07/11/2026</t>
         </is>
       </c>
-      <c r="E99" s="2" t="inlineStr">
+      <c r="E99" s="3" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="F99" s="2" t="inlineStr">
+      <c r="F99" s="3" t="inlineStr">
         <is>
           <t>2026-11-07T12:30:00-03:00</t>
         </is>
       </c>
-      <c r="G99" s="2" t="inlineStr">
+      <c r="G99" s="3" t="inlineStr">
         <is>
           <t>videos/003_skin_do_dia_coroa_suprema.mp4</t>
         </is>
       </c>
-      <c r="H99" s="2" t="inlineStr">
+      <c r="H99" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/003_skin_do_dia_coroa_suprema.mp4</t>
         </is>
       </c>
-      <c r="I99" s="2" t="inlineStr">
+      <c r="I99" s="3" t="inlineStr">
         <is>
           <t>skin do dia: Coroa Suprema (Lendário) ✨ #shorts</t>
         </is>
@@ -5697,51 +5693,51 @@
         <is>
           <t>skin do dia: Coroa Suprema (Lendário) ✨
 30 jogos no celular e no PC 🔗 kavixbrasil.com.br
-#kavix #kavixarcade #explore #trend #fyp #roblox #robloxedit #robloxfyp #gamerbrasil #mobilegames #shorts</t>
-        </is>
-      </c>
-      <c r="K99" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #foryou #viral #explore #trend #fyp #robloxedit #robloxfyp #gamerbrasil #shorts</t>
+        </is>
+      </c>
+      <c r="K99" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n">
+      <c r="A100" s="3" t="n">
         <v>99</v>
       </c>
-      <c r="B100" s="2" t="n">
+      <c r="B100" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C100" s="2" t="n">
+      <c r="C100" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="D100" s="2" t="inlineStr">
+      <c r="D100" s="3" t="inlineStr">
         <is>
           <t>07/11/2026</t>
         </is>
       </c>
-      <c r="E100" s="2" t="inlineStr">
+      <c r="E100" s="3" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F100" s="2" t="inlineStr">
+      <c r="F100" s="3" t="inlineStr">
         <is>
           <t>2026-11-07T17:00:00-03:00</t>
         </is>
       </c>
-      <c r="G100" s="2" t="inlineStr">
+      <c r="G100" s="3" t="inlineStr">
         <is>
           <t>videos/002_meme_bateria.mp4</t>
         </is>
       </c>
-      <c r="H100" s="2" t="inlineStr">
+      <c r="H100" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/002_meme_bateria.mp4</t>
         </is>
       </c>
-      <c r="I100" s="2" t="inlineStr">
+      <c r="I100" s="3" t="inlineStr">
         <is>
           <t>bateria 5% / eu tentando bater o recorde: 😭 #shorts</t>
         </is>
@@ -5750,51 +5746,51 @@
         <is>
           <t>bateria 5% / eu tentando bater o recorde: 😭
 Cria tua conta grátis e ganha itens exclusivos 🎁 link na bio
-#kavix #kavixarcade #foryou #trend #viralvideo #robloxbrasil #robloxfyp #minigames #mobilegames #shorts</t>
-        </is>
-      </c>
-      <c r="K100" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #foryou #trend #viralvideo #robloxbrasil #robloxfyp #minigames #shorts</t>
+        </is>
+      </c>
+      <c r="K100" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n">
+      <c r="A101" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="B101" s="2" t="n">
+      <c r="B101" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C101" s="2" t="n">
+      <c r="C101" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="D101" s="2" t="inlineStr">
+      <c r="D101" s="3" t="inlineStr">
         <is>
           <t>07/11/2026</t>
         </is>
       </c>
-      <c r="E101" s="2" t="inlineStr">
+      <c r="E101" s="3" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="F101" s="2" t="inlineStr">
+      <c r="F101" s="3" t="inlineStr">
         <is>
           <t>2026-11-07T20:30:00-03:00</t>
         </is>
       </c>
-      <c r="G101" s="2" t="inlineStr">
+      <c r="G101" s="3" t="inlineStr">
         <is>
           <t>videos/001_desafio_escudo.mp4</t>
         </is>
       </c>
-      <c r="H101" s="2" t="inlineStr">
+      <c r="H101" s="3" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/joaopx20-source/automaton/claude/kavix-promotional-videos-e6f1vd/promo/kavix/campanha2/videos/001_desafio_escudo.mp4</t>
         </is>
       </c>
-      <c r="I101" s="2" t="inlineStr">
+      <c r="I101" s="3" t="inlineStr">
         <is>
           <t>DESAFIO: faz 30 pontos no Escudo 😤 quem passar é lenda 👑 #shorts</t>
         </is>
@@ -5803,10 +5799,10 @@
         <is>
           <t>DESAFIO: faz 30 pontos no Escudo 😤 quem passar é lenda 👑
 Sem baixar nada: abre kavixbrasil.com.br e joga 🎮
-#kavix #kavixarcade #fyp #foryou #trend #roblox #robloxedit #robloxfyp #mobilegames #jogosdecelular #shorts</t>
-        </is>
-      </c>
-      <c r="K101" s="2" t="inlineStr">
+#kavix #kavixarcade #roblox #jogosonline #jogos #mobile #viral #fyp #foryou #trend #robloxedit #robloxfyp #mobilegames #jogosdecelular #shorts</t>
+        </is>
+      </c>
+      <c r="K101" s="3" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>

</xml_diff>